<commit_message>
Add leading and trailing space to test data.
</commit_message>
<xml_diff>
--- a/src/test/resources/se/simonsoft/cms/indexing/keydef/Techdata1-multiplekey.xlsx
+++ b/src/test/resources/se/simonsoft/cms/indexing/keydef/Techdata1-multiplekey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/takesson/git/cms-indexing-keydef/src/test/resources/se/simonsoft/cms/indexing/keydef/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C5D5AF-69B2-D54C-BC41-B44CB1E57AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8605739F-F608-B545-83A0-ABB18947D0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2040" yWindow="820" windowWidth="28200" windowHeight="17600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,12 +83,6 @@
     <t>stuff</t>
   </si>
   <si>
-    <t>WorkWidth</t>
-  </si>
-  <si>
-    <t>TransportWidth</t>
-  </si>
-  <si>
     <t>TransportHeight</t>
   </si>
   <si>
@@ -130,6 +124,12 @@
   </si>
   <si>
     <t>DeprecatedLength Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> WorkWidth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TransportWidth </t>
   </si>
 </sst>
 </file>
@@ -480,82 +480,82 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B2" s="4">
         <v>6000</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>3.2</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>2.9</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5">
         <v>3.2</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <f>B3*B5</f>
         <v>10.240000000000002</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2">
         <v>42429</v>
@@ -574,10 +574,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
@@ -597,7 +597,7 @@
     <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="6"/>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>